<commit_message>
Rename track to suite
functional and regression are suites, as a QA team says: the case field, the
review sheet column, the trace and the command (qa-agent suite TC010 functional).
A team's own sheet may still call the column Track on import.
</commit_message>
<xml_diff>
--- a/examples/bookings-team/review/cases.xlsx
+++ b/examples/bookings-team/review/cases.xlsx
@@ -504,7 +504,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Track</t>
+          <t>Suite</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -1725,7 +1725,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2. You may change Title, Criteria, Priority, Track and Tags. Steps are changed in the case file.</t>
+          <t>2. You may change Title, Criteria, Priority, Suite and Tags. Steps are changed in the case file.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Suites in the README: functional, regression, sanity, by priority
One table with what each suite is, how a case gets there and the command in
both frameworks; sanity is a tag, so a case can be regression and sanity at
once. The bookings example tags a cancellation case sanity, and run_all.sh
prints what -m regression, sanity and p0 pick, and checks that -Dgroups=p0
runs the P0 tests in Java.
</commit_message>
<xml_diff>
--- a/examples/bookings-team/review/cases.xlsx
+++ b/examples/bookings-team/review/cases.xlsx
@@ -667,7 +667,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>boundary</t>
+          <t>boundary, sanity</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -1714,7 +1714,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1750,7 +1749,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
A changed row in a case's data file sends the case back to review
The fingerprint covered the data file's name only, so editing an expected
result in the CSV after approval went unnoticed. It now covers the
file's contents too (line endings aside). The two data-driven cases in
the bookings example are re-stamped: their data files haven't changed
since they were approved (20-10-2026 and 21-10-2026).
</commit_message>
<xml_diff>
--- a/examples/bookings-team/review/cases.xlsx
+++ b/examples/bookings-team/review/cases.xlsx
@@ -701,7 +701,7 @@
       <c r="O3" s="4" t="n"/>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>9f56fb7f690a</t>
+          <t>a761a34a4590</t>
         </is>
       </c>
     </row>
@@ -1618,7 +1618,7 @@
       <c r="O15" s="4" t="n"/>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>73683198e071</t>
+          <t>1fdf4e01a987</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Data files: the rows decide approval, not the bytes, and Excel's encodings are read
- a data file saved again by Excel (or with a byte-order mark) keeps its cases approved
- data files are read as UTF-8 with or without the byte-order mark, or Windows' own encoding
- a missing data file is one error in check, not also a changed approval
</commit_message>
<xml_diff>
--- a/examples/bookings-team/review/cases.xlsx
+++ b/examples/bookings-team/review/cases.xlsx
@@ -701,7 +701,7 @@
       <c r="O3" s="4" t="n"/>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>a761a34a4590</t>
+          <t>c21f958eed76</t>
         </is>
       </c>
     </row>
@@ -1618,7 +1618,7 @@
       <c r="O15" s="4" t="n"/>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>1fdf4e01a987</t>
+          <t>393900bcbef7</t>
         </is>
       </c>
     </row>
@@ -1800,6 +1800,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1835,6 +1836,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>

</xml_diff>